<commit_message>
Sync Excel spreadsheet with current listing data
</commit_message>
<xml_diff>
--- a/Team Utah Commercial Listings.xlsx
+++ b/Team Utah Commercial Listings.xlsx
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -547,7 +547,7 @@
           <t>Res. Land</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="n">
         <v>1.52</v>
       </c>
@@ -570,12 +570,12 @@
           <t>https://www.crexi.com/properties/2140992/utah-6-lots-on-jordan-canal-rd</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n"/>
+      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>8987 Magna Main St</t>
+          <t>8979 W Magna Main St</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
@@ -589,13 +589,15 @@
         </is>
       </c>
       <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
+      <c r="E3" s="4" t="n">
+        <v>1975</v>
+      </c>
       <c r="F3" s="5" t="n">
-        <v>1150000</v>
+        <v>500000</v>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>photos/magna-main-8987/1-auto-from-realnex.jpg</t>
+          <t>photos/magna-main-8979/MM Restaurant sm.jpg</t>
         </is>
       </c>
       <c r="H3" s="4" t="inlineStr">
@@ -605,137 +607,141 @@
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/properties/2213430/utah-8987-w-magna-main-bar-restaurant-entertainment</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>https://www.loopnet.com/Listing/8987-W-Magna-Main-St-Magna-UT/38108070/</t>
-        </is>
-      </c>
+          <t>https://www.crexi.com/properties/2352359/utah-magna-main-restaurant</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>1366 N Main St, Layton 84041</t>
+          <t>8987 Magna Main St</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Retail Land</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="E4" s="2" t="n"/>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Under Contract</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n">
+        <v>5925</v>
+      </c>
       <c r="F4" s="3" t="n">
-        <v>2550000</v>
+        <v>1150000</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>photos/layton-main/1-auto-from-wfrmls.jpg</t>
+          <t>photos/magna-main-8987/1-auto-from-realnex.jpg</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://marketedge.realnex.com/ePublish.aspx?propid=167412-1</t>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169469-1</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/properties/1940627/utah-layton-mainstreet</t>
+          <t>https://www.crexi.com/properties/2213430/utah-8987-w-magna-main-bar-restaurant-entertainment</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>https://www.loopnet.com/Listing/1366-Main-St-Layton-UT/36053699/</t>
+          <t>https://www.loopnet.com/Listing/8987-W-Magna-Main-St-Magna-UT/38108070/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2955 E 3500 S, Delta - Stefanoff Farms</t>
+          <t>1366 N Main St, Layton 84041</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Ag. Land</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
+          <t>Retail Land</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Under Contract</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>2.02</v>
+      </c>
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="5" t="n">
-        <v>75000000</v>
+        <v>2550000</v>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>photos/stefanoff-farms/0124332c613d48c1a066d3b7d19b60c6_3000x2000_resize (1).jpg</t>
+          <t>photos/layton-main/1-auto-from-wfrmls.jpg</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>https://marketedge.realnex.com/ePublish.aspx?propid=165613-1</t>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=167412-1</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/properties/2305853/utah-delta-land-water</t>
+          <t>https://www.crexi.com/properties/1940627/utah-layton-mainstreet</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>https://www.loopnet.com/Listing/2955-E-3500-S-Delta-UT/39195100/</t>
+          <t>https://www.loopnet.com/Listing/1366-Main-St-Layton-UT/36053699/</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>851 N McCormick Way</t>
+          <t>2955 E 3500 S, Delta, UT</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n"/>
+          <t>Ag. Land</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="n">
-        <v>1.5</v>
+        <v>2776</v>
       </c>
       <c r="E6" s="2" t="n"/>
-      <c r="F6" s="3" t="n">
-        <v>5115000</v>
-      </c>
+      <c r="F6" s="3" t="n"/>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>photos/mccormick-851/1-auto-from-realnex.jpg</t>
+          <t>photos/stefanoff-farms/0124332c613d48c1a066d3b7d19b60c6_3000x2000_resize (1).jpg</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169863-1</t>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=165613-1</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/properties/2311859/utah-851-mccormick-way</t>
+          <t>https://www.crexi.com/properties/2305853/utah-delta-land-water</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>https://www.loopnet.com/Listing/851-N-McCormick-Way-Layton-UT/39242904/</t>
+          <t>https://www.loopnet.com/Listing/2955-E-3500-S-Delta-UT/39195100/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>855 N McCormick Way</t>
+          <t>851 N McCormick Way</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
@@ -743,17 +749,17 @@
           <t>Industrial</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n"/>
+      <c r="C7" s="4" t="inlineStr"/>
       <c r="D7" s="4" t="n">
         <v>1.5</v>
       </c>
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="5" t="n">
-        <v>3825000</v>
+        <v>5115000</v>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>photos/mccormick-855/1-auto-from-realnex.jpg</t>
+          <t>photos/mccormick-851/1-auto-from-realnex.jpg</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
@@ -763,55 +769,59 @@
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/properties/2311860/utah-855-mccormick</t>
+          <t>https://www.crexi.com/properties/2311859/utah-851-mccormick-way</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>https://www.loopnet.com/Listing/855-McCormick-Way-Layton-UT/39243024/</t>
+          <t>https://www.loopnet.com/Listing/851-N-McCormick-Way-Layton-UT/39242904/</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>1295 E Belladonna Dr</t>
+          <t>855 N McCormick Way</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Industrial Land</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n"/>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="n">
-        <v>0.84</v>
+        <v>1.5</v>
       </c>
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="3" t="n">
-        <v>1221858</v>
+        <v>3825000</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>photos/belladonna-1295/1-auto-from-realnex.jpg</t>
+          <t>photos/mccormick-855/1-auto-from-realnex.jpg</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169863-1</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/properties/2313320/utah-306-sweetwater-industrial</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="n"/>
+          <t>https://www.crexi.com/properties/2311860/utah-855-mccormick</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.loopnet.com/Listing/855-McCormick-Way-Layton-UT/39243024/</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>1448 E Jasmine St</t>
+          <t>1295 E Belladonna Dr</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -819,15 +829,17 @@
           <t>Industrial Land</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n"/>
-      <c r="D9" s="4" t="n"/>
+      <c r="C9" s="4" t="inlineStr"/>
+      <c r="D9" s="4" t="n">
+        <v>0.84</v>
+      </c>
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="5" t="n">
-        <v>1306800</v>
+        <v>329314</v>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>photos/jasmine-1448/1-auto-from-realnex.jpg</t>
+          <t>photos/belladonna-1295/1-auto-from-realnex.jpg</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -837,33 +849,33 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/properties/2313344/utah-307-sweetwater-commerical</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="n"/>
+          <t>https://www.crexi.com/properties/2313320/utah-306-sweetwater-industrial</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>1174 E Belladonna Dr</t>
+          <t>1448 E Jasmine St</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Industrial Land</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n"/>
+          <t>Office Land</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="n">
-        <v>4.21</v>
+        <v>1.96</v>
       </c>
       <c r="E10" s="2" t="n"/>
       <c r="F10" s="3" t="n">
-        <v>1650488</v>
+        <v>1280664</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>photos/belladonna-1174/1-auto-from-wfrmls.jpg</t>
+          <t>photos/jasmine-1448/1-auto-from-realnex.jpg</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -873,37 +885,33 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/properties/2313671/utah-commerical-and-industrial-site---eagle-mountian-corridor</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>https://www.loopnet.com/Listing/1174-Belladonna-dr-Eagle-Mountain-UT/38996273/</t>
-        </is>
-      </c>
+          <t>https://www.crexi.com/properties/2313344/utah-307-sweetwater-commerical</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Eagle Mountain Commercial Corridor (115.98 ac)</t>
+          <t>1174 E Belladonna Dr</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Commercial Land</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n"/>
+          <t>Industrial Land</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr"/>
       <c r="D11" s="4" t="n">
-        <v>115.98</v>
+        <v>4.21</v>
       </c>
       <c r="E11" s="4" t="n"/>
       <c r="F11" s="5" t="n">
-        <v>20218810</v>
+        <v>1650488</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>photos/eagle-mtn-corridor/1-auto-from-wfrmls.jpg</t>
+          <t>photos/belladonna-1174/1-auto-from-wfrmls.jpg</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -913,33 +921,37 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/properties/2313593/utah-11598-acre-corridor-commercial</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="n"/>
+          <t>https://www.crexi.com/properties/2313549/utah-313-sweetwater-industrial</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.loopnet.com/Listing/1174-Belladonna-dr-Eagle-Mountain-UT/38996273/</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>1900 N Piper Ln, Eagle Mountain, UT 84005</t>
+          <t>EM Commercial Corridor</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Commercial Land</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n"/>
+          <t>Industrial Data</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="n">
-        <v>106.52</v>
+        <v>90.81</v>
       </c>
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="3" t="n">
-        <v>30312533</v>
+        <v>23734102</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>photos/piper-ln/1-auto-from-wfrmls.jpg</t>
+          <t>photos/eagle-mtn-corridor/Marked ABCDE.png</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -947,141 +959,153 @@
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>https://www.crexi.com/properties/2313564/utah-106-acres-agricultural-to-develop</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>210 E Main St, American Fork, UT 84003</t>
+          <t>Eagle Mountain Commercial</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Retail Land</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Under Contract</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="n"/>
+          <t>Commercial Land</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr"/>
+      <c r="D13" s="4" t="n">
+        <v>77.36</v>
+      </c>
       <c r="E13" s="4" t="n"/>
       <c r="F13" s="5" t="n">
-        <v>2200000</v>
+        <v>20218810</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>photos/american-fork-main/7fd04a324d104428bd1b36f973012f91_3000x2000_resize.jpg</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="n"/>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>https://www.crexi.com/properties/2432043/utah-210-e-main-street</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="n"/>
+          <t>photos/eagle-mtn-corridor/1-auto-from-wfrmls.jpg</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>512 E Larchwood Dr, Midvale, UT 84121</t>
+          <t>1900 N Piper Ln, Eagle Mountain</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Income</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
+          <t>Industrial Land</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="n">
+        <v>115.96</v>
+      </c>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="3" t="n">
-        <v>700000</v>
+        <v>30312533</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>photos/larchwood-512/17c0475d6a9b410687cc8db121fd356d_3000x2000_resize.jpg</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n"/>
+          <t>photos/piper-ln/1-auto-from-wfrmls.jpg</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
+        </is>
+      </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/properties/2253599/utah-non-conforming-midvale-duplex-w-separate-meters</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="n"/>
+          <t>https://www.crexi.com/properties/2313593/utah-11598-acre-corridor-commercial</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>1213 E Belladonna Dr</t>
+          <t>210 E Main St, American Fork, UT</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Industrial Land</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="n"/>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Under Contract</t>
+        </is>
+      </c>
       <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
+      <c r="E15" s="4" t="n">
+        <v>4994</v>
+      </c>
       <c r="F15" s="5" t="n">
-        <v>341075</v>
+        <v>2200000</v>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>photos/belladonna-1213/1213 E.png</t>
+          <t>photos/american-fork-main/7fd04a324d104428bd1b36f973012f91_3000x2000_resize.jpg</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="n"/>
-      <c r="J15" s="4" t="n"/>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169633-1</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.crexi.com/properties/2432043/utah-210-e-main-street</t>
+        </is>
+      </c>
+      <c r="J15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>1239 E Belladonna Dr</t>
+          <t>512 E Larchwood Dr, Midvale, UT</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Industrial Land</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="n"/>
+          <t>Income</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
+      <c r="E16" s="2" t="n">
+        <v>2456</v>
+      </c>
       <c r="F16" s="3" t="n">
-        <v>329314</v>
+        <v>700000</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>photos/belladonna-1239/1239 E.png</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="n"/>
+          <t>photos/larchwood-512/17c0475d6a9b410687cc8db121fd356d_3000x2000_resize.jpg</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.crexi.com/properties/2253599/utah-non-conforming-midvale-duplex-w-separate-meters</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>1267 E Belladonna Dr</t>
+          <t>1213 E Belladonna Dr</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -1089,15 +1113,17 @@
           <t>Industrial Land</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
+      <c r="C17" s="4" t="inlineStr"/>
+      <c r="D17" s="4" t="n">
+        <v>0.87</v>
+      </c>
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="5" t="n">
-        <v>1280664</v>
+        <v>341075</v>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>photos/belladonna-1267/1267 E.png</t>
+          <t>photos/belladonna-1213/1213 E.png</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1105,13 +1131,13 @@
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I17" s="4" t="n"/>
-      <c r="J17" s="4" t="n"/>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>1394 E Jasmine St</t>
+          <t>1239 E Belladonna Dr</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1119,15 +1145,17 @@
           <t>Industrial Land</t>
         </is>
       </c>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="n">
+        <v>0.87</v>
+      </c>
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="3" t="n">
-        <v>929135</v>
+        <v>341075</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>photos/jasmine-1394/1394 E.png</t>
+          <t>photos/belladonna-1239/1239 E.png</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1135,13 +1163,13 @@
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>1344 E Jasmine St</t>
+          <t>1267 E Belladonna Dr</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
@@ -1149,15 +1177,17 @@
           <t>Industrial Land</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n"/>
-      <c r="D19" s="4" t="n"/>
+      <c r="C19" s="4" t="inlineStr"/>
+      <c r="D19" s="4" t="n">
+        <v>0.87</v>
+      </c>
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="5" t="n">
-        <v>1306800</v>
+        <v>341075</v>
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>photos/jasmine-1344/1344 E.png</t>
+          <t>photos/belladonna-1267/1267 E.png</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -1165,29 +1195,31 @@
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I19" s="4" t="n"/>
-      <c r="J19" s="4" t="n"/>
+      <c r="I19" s="4" t="inlineStr"/>
+      <c r="J19" s="4" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2694 N Peony St</t>
+          <t>1394 E Jasmine St</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Industrial Land</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
+          <t>Commercial Land</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="n">
+        <v>1.87</v>
+      </c>
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="3" t="n">
-        <v>929135</v>
+        <v>1221858</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>photos/peony-2694/2694 N.png</t>
+          <t>photos/jasmine-1394/1394 E.png</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1195,13 +1227,13 @@
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>1290 E Belladonna Dr</t>
+          <t>1344 E Jasmine St</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
@@ -1209,17 +1241,17 @@
           <t>Industrial Land</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n"/>
+      <c r="C21" s="4" t="inlineStr"/>
       <c r="D21" s="4" t="n">
-        <v>4.21</v>
+        <v>2</v>
       </c>
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="5" t="n">
-        <v>976180</v>
+        <v>1306800</v>
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>photos/belladonna-1290/1-auto-from-wfrmls.jpg</t>
+          <t>photos/jasmine-1344/1344 E.png</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -1227,13 +1259,13 @@
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I21" s="4" t="n"/>
-      <c r="J21" s="4" t="n"/>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>1232 E Belladonna Dr</t>
+          <t>2694 N Peony St</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1241,17 +1273,17 @@
           <t>Industrial Land</t>
         </is>
       </c>
-      <c r="C22" s="2" t="n"/>
+      <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="n">
-        <v>77.36</v>
+        <v>2.37</v>
       </c>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="3" t="n">
-        <v>1642648</v>
+        <v>929135</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>photos/belladonna-1232/1232 E Belladona.png</t>
+          <t>photos/peony-2694/2694 N.png</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1259,70 +1291,142 @@
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I22" s="2" t="n"/>
-      <c r="J22" s="2" t="n"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>2900 N Pony Express Pkwy</t>
+          <t>1290 E Belladonna Dr</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Commercial Land</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="n"/>
+          <t>Industrial Land</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr"/>
       <c r="D23" s="4" t="n">
-        <v>90.81</v>
+        <v>2.49</v>
       </c>
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="5" t="n">
-        <v>18028613</v>
-      </c>
-      <c r="G23" s="4" t="n"/>
+        <v>976180</v>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>photos/belladonna-1290/1-auto-from-wfrmls.jpg</t>
+        </is>
+      </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>https://www.crexi.com/properties/2313671/utah-commerical-and-industrial-site---eagle-mountian-corridor</t>
-        </is>
-      </c>
-      <c r="J23" s="4" t="n"/>
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>3000 Lake Mountain Rd</t>
+          <t>1232 E Belladonna Dr</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Commercial Land</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
+          <t>Industrial Land</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="n">
+        <v>4.19</v>
+      </c>
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="3" t="n">
+        <v>1642648</v>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>photos/belladonna-1232/1232 E Belladona.png</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2900 N Pony Express Pkwy</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Commercial Land</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>69.98</v>
+      </c>
+      <c r="F25" t="n">
+        <v>18028613</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>photos/pony-express-2900/43751716da6f413396a066ecaccf9783_3000x2000_resize (1).jpg</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>https://www.crexi.com/properties/2313671/utah-commerical-and-industrial-site---eagle-mountian-corridor</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>3000 Lake Mountain Rd</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Ag. Land</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>106.52</v>
+      </c>
+      <c r="F26" t="n">
         <v>27840067</v>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>photos/lake-mountain-3000/916a4f043bee4e10a7ff3b011200f30b_3000x2000_resize (1).jpg</t>
         </is>
       </c>
-      <c r="H24" s="2" t="n"/>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2313564/utah-106-acres-agricultural-to-develop</t>
         </is>
       </c>
-      <c r="J24" s="2" t="n"/>
+      <c r="J26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1405,19 +1509,21 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2464 W 12600 South #160-170 (min 3yr)</t>
+          <t>2464 W 12600 South #160-170</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Office</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n"/>
+          <t>Retail</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
+      <c r="E2" s="2" t="n">
+        <v>3102</v>
+      </c>
       <c r="F2" s="6" t="n">
-        <v>16.5</v>
+        <v>22</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -1426,7 +1532,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://marketedge.realnex.com/ePublish.aspx?propid=172543-1</t>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=165263-1</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -1434,7 +1540,7 @@
           <t>https://www.crexi.com/lease/properties/194684/utah-riverton-retail-center</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n"/>
+      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1447,9 +1553,11 @@
           <t>Office</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n"/>
+      <c r="C3" s="4" t="inlineStr"/>
       <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
+      <c r="E3" s="4" t="n">
+        <v>1320</v>
+      </c>
       <c r="F3" s="7" t="n">
         <v>14.5</v>
       </c>
@@ -1458,13 +1566,17 @@
           <t>photos/lease-ogden/fe4c4f2505b0423aab153df998a526be_3000x2000_resize (1).jpg</t>
         </is>
       </c>
-      <c r="H3" s="4" t="n"/>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=165807-1</t>
+        </is>
+      </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
           <t>https://www.crexi.com/lease/properties/968935/utah-1673-w-2650-s-office</t>
         </is>
       </c>
-      <c r="J3" s="4" t="n"/>
+      <c r="J3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1474,12 +1586,14 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Industrial</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n"/>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
+      <c r="E4" s="2" t="n">
+        <v>2300</v>
+      </c>
       <c r="F4" s="6" t="n">
         <v>16.5</v>
       </c>
@@ -1488,13 +1602,17 @@
           <t>photos/lease-9489-6400w/4bc876872cd0486b88beb7122754de70_3000x2000_resize.jpg</t>
         </is>
       </c>
-      <c r="H4" s="2" t="n"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=172543-1</t>
+        </is>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>https://www.crexi.com/lease/properties/1130679/utah-9489-south-6400-west-west-jordan-ut-84081</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n"/>
+      <c r="J4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1507,8 +1625,10 @@
           <t>Retail</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
+      <c r="C5" s="4" t="inlineStr"/>
+      <c r="D5" s="4" t="n">
+        <v>1.81</v>
+      </c>
       <c r="E5" s="4" t="n"/>
       <c r="F5" s="4" t="n"/>
       <c r="G5" s="4" t="inlineStr">
@@ -1516,13 +1636,13 @@
           <t>photos/lease-3666-state/d3d12a3340794645ba0032a9c30ca3f4_3000x2000_resize (1).jpg</t>
         </is>
       </c>
-      <c r="H5" s="4" t="n"/>
+      <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="4" t="inlineStr">
         <is>
           <t>https://www.crexi.com/lease/properties/949135/utah-state-street-retail-pads</t>
         </is>
       </c>
-      <c r="J5" s="4" t="n"/>
+      <c r="J5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1535,9 +1655,11 @@
           <t>Industrial</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n"/>
+      <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
+      <c r="E6" s="2" t="n">
+        <v>10000</v>
+      </c>
       <c r="F6" s="6" t="n">
         <v>15</v>
       </c>
@@ -1546,7 +1668,11 @@
           <t>photos/lease-5918-350w/b3149d9d10d949989fa3b854043c9e2c_3000x2000_resize.jpg</t>
         </is>
       </c>
-      <c r="H6" s="2" t="n"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=172198-1</t>
+        </is>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>https://www.crexi.com/lease/properties/1108954/utah-murray-industrial</t>
@@ -1647,39 +1773,59 @@
           <t>Office</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
+      <c r="E2" s="2" t="n">
+        <v>4661</v>
+      </c>
       <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>photos/1755/IMG_8966-EDIT.jpg</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=166547-1</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>3600 N Fairfield, Layton - Kihomac</t>
+          <t>3600 N Fairfield, East Gate HAFB</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Office</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
+          <t>Industrial Land</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr"/>
+      <c r="D3" s="4" t="n">
+        <v>10.08</v>
+      </c>
       <c r="E3" s="4" t="n"/>
       <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="4" t="n"/>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>photos/kihomac-fairfield/Aerial with HAFB and parcels.png</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=149090-1</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr"/>
+      <c r="J3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>205 W 700 South - CMN</t>
+          <t>205 W 700 South - CMN, SLC</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -1687,62 +1833,88 @@
           <t>Office</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n"/>
+      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
+      <c r="E4" s="2" t="n">
+        <v>43290</v>
+      </c>
       <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>photos/cmn-700-south/pdl23tp.jpeg</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>https://marketedge.realnex.com/ePublish.aspx?propid=168914-1</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>1701 S 5350 W</t>
+          <t>1701 S 5350 W, SLC</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n"/>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Leased</t>
+        </is>
+      </c>
       <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
+      <c r="E5" s="4" t="n">
+        <v>18000</v>
+      </c>
       <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>photos/1701-5350w/1701-exterior.png</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=164739-1</t>
         </is>
       </c>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="n"/>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Bridger Rd</t>
+          <t>2608 Bridger Rd, SLC</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Commercial</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n"/>
+          <t>Industrial</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
+      <c r="E6" s="2" t="n">
+        <v>24248</v>
+      </c>
       <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>photos/bridger-rd/0.jpg</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=156299-1</t>
         </is>
       </c>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Regenerate spreadsheet from current real-listings.json
</commit_message>
<xml_diff>
--- a/Team Utah Commercial Listings.xlsx
+++ b/Team Utah Commercial Listings.xlsx
@@ -39,7 +39,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A365D"/>
+        <fgColor rgb="001A3C64"/>
       </patternFill>
     </fill>
   </fills>
@@ -425,76 +425,82 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
-    <col width="55" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
     <col width="50" customWidth="1" min="11" max="11"/>
+    <col width="50" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Address</t>
+          <t>address</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>type</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>section</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>status</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Acres</t>
+          <t>acres</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>acresDisplay</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>sf</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>OM Link</t>
+          <t>price</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Crexi Link</t>
+          <t>photo</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>LoopNet Link</t>
+          <t>om</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Photo Path</t>
+          <t>crexi</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>loopnet</t>
         </is>
       </c>
     </row>
@@ -519,25 +525,25 @@
         <v>1.52</v>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>1300000</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>photos/jordan-canal/1-auto-from-realnex.jpg</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=168633-1</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2140992/utah-6-lots-on-jordan-canal-rd</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>photos/jordan-canal/1-auto-from-realnex.jpg</t>
-        </is>
-      </c>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -560,29 +566,29 @@
           <t>Under Contract</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="n">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="n">
         <v>1975</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>500000</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>photos/magna-main-8979/MM Restaurant sm.jpg</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169469-1</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2352359/utah-magna-main-restaurant</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>photos/magna-main-8979/MM Restaurant sm.jpg</t>
-        </is>
-      </c>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -605,31 +611,31 @@
           <t>Under Contract</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="n">
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="n">
         <v>5925</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>1150000</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>photos/magna-main-8987/1-auto-from-realnex.jpg</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169469-1</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2213430/utah-8987-w-magna-main-bar-restaurant-entertainment</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>https://www.loopnet.com/Listing/8987-W-Magna-Main-St-Magna-UT/38108070/</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>photos/magna-main-8987/1-auto-from-realnex.jpg</t>
         </is>
       </c>
     </row>
@@ -658,27 +664,27 @@
         <v>2.02</v>
       </c>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>2550000</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>photos/layton-main/1-auto-from-wfrmls.jpg</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=167412-1</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/1940627/utah-layton-mainstreet</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>https://www.loopnet.com/Listing/1366-Main-St-Layton-UT/36053699/</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>photos/layton-main/1-auto-from-wfrmls.jpg</t>
         </is>
       </c>
     </row>
@@ -699,31 +705,32 @@
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
+      <c r="E6" t="n">
+        <v>2776</v>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>2,776 W/water</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>photos/stefanoff-farms/0124332c613d48c1a066d3b7d19b60c6_3000x2000_resize (1).jpg</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=165613-1</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2305853/utah-delta-land-water</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>https://www.loopnet.com/Listing/2955-E-3500-S-Delta-UT/39195100/</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>photos/stefanoff-farms/0124332c613d48c1a066d3b7d19b60c6_3000x2000_resize (1).jpg</t>
         </is>
       </c>
     </row>
@@ -748,27 +755,27 @@
         <v>1.5</v>
       </c>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" t="n">
+      <c r="H7" t="n">
         <v>5115000</v>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>photos/mccormick-851/1-auto-from-realnex.jpg</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169863-1</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2311859/utah-851-mccormick-way</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>https://www.loopnet.com/Listing/851-N-McCormick-Way-Layton-UT/39242904/</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>photos/mccormick-851/1-auto-from-realnex.jpg</t>
         </is>
       </c>
     </row>
@@ -793,27 +800,27 @@
         <v>1.5</v>
       </c>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="n">
+      <c r="H8" t="n">
         <v>3825000</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>photos/mccormick-855/1-auto-from-realnex.jpg</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169863-1</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2311860/utah-855-mccormick</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>https://www.loopnet.com/Listing/855-McCormick-Way-Layton-UT/39243024/</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>photos/mccormick-855/1-auto-from-realnex.jpg</t>
         </is>
       </c>
     </row>
@@ -838,25 +845,25 @@
         <v>0.84</v>
       </c>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="n">
+      <c r="H9" t="n">
         <v>329314</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>photos/belladonna-1295/1-auto-from-realnex.jpg</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2313320/utah-306-sweetwater-industrial</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>photos/belladonna-1295/1-auto-from-realnex.jpg</t>
-        </is>
-      </c>
+      <c r="L9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -879,25 +886,25 @@
         <v>1.96</v>
       </c>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>1280664</v>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>photos/jasmine-1448/1-auto-from-realnex.jpg</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2313344/utah-307-sweetwater-commerical</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>photos/jasmine-1448/1-auto-from-realnex.jpg</t>
-        </is>
-      </c>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -920,27 +927,27 @@
         <v>4.21</v>
       </c>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>1650488</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>photos/belladonna-1174/1-auto-from-wfrmls.jpg</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2313549/utah-313-sweetwater-industrial</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>https://www.loopnet.com/Listing/1174-Belladonna-dr-Eagle-Mountain-UT/38996273/</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>photos/belladonna-1174/1-auto-from-wfrmls.jpg</t>
         </is>
       </c>
     </row>
@@ -965,21 +972,21 @@
         <v>90.81</v>
       </c>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>23734102</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>photos/eagle-mtn-corridor/marked-abcde.png</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>photos/eagle-mtn-corridor/marked-abcde.png</t>
-        </is>
-      </c>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1002,21 +1009,21 @@
         <v>77.36</v>
       </c>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>20218810</v>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>photos/eagle-mtn-corridor/marked-abcde.png</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>photos/eagle-mtn-corridor/marked-abcde.png</t>
-        </is>
-      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1039,25 +1046,25 @@
         <v>115.96</v>
       </c>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>30312533</v>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>photos/piper-ln/1-auto-from-wfrmls.jpg</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2313593/utah-11598-acre-corridor-commercial</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>photos/piper-ln/1-auto-from-wfrmls.jpg</t>
-        </is>
-      </c>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1080,29 +1087,29 @@
           <t>Under Contract</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="n">
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="n">
         <v>4994</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>2200000</v>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>photos/american-fork-main/7fd04a324d104428bd1b36f973012f91_3000x2000_resize.jpg</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169633-1</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2432043/utah-210-e-main-street</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>photos/american-fork-main/7fd04a324d104428bd1b36f973012f91_3000x2000_resize.jpg</t>
-        </is>
-      </c>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1121,25 +1128,25 @@
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="n">
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="n">
         <v>2456</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>700000</v>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/properties/2253599/utah-non-conforming-midvale-duplex-w-separate-meters</t>
+          <t>photos/larchwood-512/17c0475d6a9b410687cc8db121fd356d_3000x2000_resize.jpg</t>
         </is>
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
-          <t>photos/larchwood-512/17c0475d6a9b410687cc8db121fd356d_3000x2000_resize.jpg</t>
-        </is>
-      </c>
+          <t>https://www.crexi.com/properties/2253599/utah-non-conforming-midvale-duplex-w-separate-meters</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1162,21 +1169,21 @@
         <v>0.87</v>
       </c>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>341075</v>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>photos/belladonna-1213/1213 E.png</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>photos/belladonna-1213/1213 E.png</t>
-        </is>
-      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1199,21 +1206,21 @@
         <v>0.87</v>
       </c>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>341075</v>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>photos/belladonna-1239/1239 E.png</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>photos/belladonna-1239/1239 E.png</t>
-        </is>
-      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1236,21 +1243,21 @@
         <v>0.87</v>
       </c>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>341075</v>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>photos/belladonna-1267/1267 E.png</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>photos/belladonna-1267/1267 E.png</t>
-        </is>
-      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1273,21 +1280,21 @@
         <v>1.87</v>
       </c>
       <c r="F20" t="inlineStr"/>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>1221858</v>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>photos/jasmine-1394/1394 E.png</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>photos/jasmine-1394/1394 E.png</t>
-        </is>
-      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1310,21 +1317,21 @@
         <v>2</v>
       </c>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>1306800</v>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>photos/jasmine-1344/1344 E.png</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>photos/jasmine-1344/1344 E.png</t>
-        </is>
-      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1347,21 +1354,21 @@
         <v>2.37</v>
       </c>
       <c r="F22" t="inlineStr"/>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>929135</v>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>photos/peony-2694/2694 N.png</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>photos/peony-2694/2694 N.png</t>
-        </is>
-      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1384,21 +1391,21 @@
         <v>2.49</v>
       </c>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="n">
+      <c r="H23" t="n">
         <v>976180</v>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>photos/belladonna-1290/1-auto-from-wfrmls.jpg</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>photos/belladonna-1290/1-auto-from-wfrmls.jpg</t>
-        </is>
-      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1421,21 +1428,21 @@
         <v>4.19</v>
       </c>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" t="n">
+      <c r="H24" t="n">
         <v>1642648</v>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>photos/belladonna-1232/1232 E Belladona.png</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>photos/belladonna-1232/1232 E Belladona.png</t>
-        </is>
-      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1458,25 +1465,25 @@
         <v>69.98</v>
       </c>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" t="n">
+      <c r="H25" t="n">
         <v>18028613</v>
       </c>
-      <c r="H25" t="inlineStr">
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>photos/pony-express-2900/43751716da6f413396a066ecaccf9783_3000x2000_resize (1).jpg</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2313671/utah-commerical-and-industrial-site---eagle-mountian-corridor</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>photos/pony-express-2900/43751716da6f413396a066ecaccf9783_3000x2000_resize (1).jpg</t>
-        </is>
-      </c>
+      <c r="L25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1499,25 +1506,25 @@
         <v>106.52</v>
       </c>
       <c r="F26" t="inlineStr"/>
-      <c r="G26" t="n">
+      <c r="H26" t="n">
         <v>27840067</v>
       </c>
-      <c r="H26" t="inlineStr">
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>photos/lake-mountain-3000/916a4f043bee4e10a7ff3b011200f30b_3000x2000_resize (1).jpg</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=169603-1</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>https://www.crexi.com/properties/2313564/utah-106-acres-agricultural-to-develop</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>photos/lake-mountain-3000/916a4f043bee4e10a7ff3b011200f30b_3000x2000_resize (1).jpg</t>
-        </is>
-      </c>
+      <c r="L26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1536,31 +1543,29 @@
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="n">
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="n">
         <v>3102</v>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>$22.00/SF/yr</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
+      <c r="H27" t="n">
+        <v>22</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>photos/lease-12600-south/14d79802da3345f99ab333f8a0e6761c_3000x2000_resize.jpg</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=165263-1</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>https://www.crexi.com/lease/properties/194684/utah-riverton-retail-center</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>photos/lease-12600-south/14d79802da3345f99ab333f8a0e6761c_3000x2000_resize.jpg</t>
-        </is>
-      </c>
+      <c r="L27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1579,31 +1584,29 @@
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="n">
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="n">
         <v>1320</v>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>$14.50/SF/yr</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
+      <c r="H28" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>photos/lease-ogden/fe4c4f2505b0423aab153df998a526be_3000x2000_resize (1).jpg</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=165807-1</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>https://www.crexi.com/lease/properties/968935/utah-1673-w-2650-s-office</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>photos/lease-ogden/fe4c4f2505b0423aab153df998a526be_3000x2000_resize (1).jpg</t>
-        </is>
-      </c>
+      <c r="L28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1622,31 +1625,29 @@
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="n">
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="n">
         <v>2300</v>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>$16.50/SF/yr</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
+      <c r="H29" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>photos/lease-9489-6400w/4bc876872cd0486b88beb7122754de70_3000x2000_resize.jpg</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=172543-1</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>https://www.crexi.com/lease/properties/1130679/utah-9489-south-6400-west-west-jordan-ut-84081</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>photos/lease-9489-6400w/4bc876872cd0486b88beb7122754de70_3000x2000_resize.jpg</t>
-        </is>
-      </c>
+      <c r="L29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1669,19 +1670,18 @@
         <v>1.81</v>
       </c>
       <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>https://www.crexi.com/lease/properties/949135/utah-state-street-retail-pads</t>
+          <t>photos/lease-3666-state/d3d12a3340794645ba0032a9c30ca3f4_3000x2000_resize (1).jpg</t>
         </is>
       </c>
       <c r="J30" t="inlineStr"/>
       <c r="K30" t="inlineStr">
         <is>
-          <t>photos/lease-3666-state/d3d12a3340794645ba0032a9c30ca3f4_3000x2000_resize (1).jpg</t>
-        </is>
-      </c>
+          <t>https://www.crexi.com/lease/properties/949135/utah-state-street-retail-pads</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1700,33 +1700,31 @@
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="n">
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="n">
         <v>10000</v>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>$15.00/SF/yr</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
+      <c r="H31" t="n">
+        <v>15</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>photos/lease-5918-350w/b3149d9d10d949989fa3b854043c9e2c_3000x2000_resize.jpg</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=172198-1</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>https://www.crexi.com/lease/properties/1108954/utah-murray-industrial</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="L31" t="inlineStr">
         <is>
           <t>https://www.loopnet.com/Listing/5918-5924-S-350-W-Salt-Lake-City-UT/39433482/</t>
-        </is>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>photos/lease-5918-350w/b3149d9d10d949989fa3b854043c9e2c_3000x2000_resize.jpg</t>
         </is>
       </c>
     </row>
@@ -1747,23 +1745,22 @@
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="n">
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="n">
         <v>4661</v>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr">
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>photos/1755/IMG_8966-EDIT.jpg</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=166547-1</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>photos/1755/IMG_8966-EDIT.jpg</t>
-        </is>
-      </c>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1786,19 +1783,18 @@
         <v>10.08</v>
       </c>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr">
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>photos/kihomac-fairfield/Aerial with HAFB and parcels.png</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=149090-1</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>photos/kihomac-fairfield/Aerial with HAFB and parcels.png</t>
-        </is>
-      </c>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1817,23 +1813,22 @@
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="n">
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="n">
         <v>43290</v>
       </c>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>photos/cmn-700-south/pdl23tp.jpeg</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=168914-1</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>photos/cmn-700-south/pdl23tp.jpeg</t>
-        </is>
-      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1856,23 +1851,22 @@
           <t>Leased</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="n">
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="n">
         <v>18000</v>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr">
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>photos/1701-5350w/1701-exterior.png</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=164739-1</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>photos/1701-5350w/1701-exterior.png</t>
-        </is>
-      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1891,23 +1885,22 @@
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="n">
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="n">
         <v>24248</v>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr">
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>photos/bridger-rd/0.jpg</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
         <is>
           <t>https://marketedge.realnex.com/ePublish.aspx?propid=156299-1</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>photos/bridger-rd/0.jpg</t>
-        </is>
-      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>